<commit_message>
placas,eco y wrapper portones arreglados
</commit_message>
<xml_diff>
--- a/backend/excel/catalogo.xlsx
+++ b/backend/excel/catalogo.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="10275" tabRatio="939" firstSheet="2" activeTab="11"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="10275" tabRatio="939" firstSheet="8" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="VENTANAS_HERRERO" sheetId="1" r:id="rId1"/>
@@ -3253,7 +3253,9 @@
   <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.42578125" style="1"/>
+    <col min="2" max="2" width="21" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -3290,10 +3292,10 @@
         <v>193</v>
       </c>
       <c r="D2" s="1">
-        <v>62100</v>
+        <v>76300</v>
       </c>
       <c r="E2" s="1">
-        <v>66000</v>
+        <v>81100</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3307,10 +3309,10 @@
         <v>194</v>
       </c>
       <c r="D3" s="1">
-        <v>62100</v>
+        <v>76300</v>
       </c>
       <c r="E3" s="1">
-        <v>66000</v>
+        <v>81100</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -3324,10 +3326,10 @@
         <v>195</v>
       </c>
       <c r="D4" s="1">
-        <v>66000</v>
+        <v>81100</v>
       </c>
       <c r="E4" s="1">
-        <v>70100</v>
+        <v>86112</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3341,10 +3343,10 @@
         <v>193</v>
       </c>
       <c r="D5" s="1">
-        <v>112717</v>
+        <v>138500</v>
       </c>
       <c r="E5" s="1">
-        <v>117180</v>
+        <v>144100</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -3358,10 +3360,10 @@
         <v>194</v>
       </c>
       <c r="D6" s="1">
-        <v>112717</v>
+        <v>138500</v>
       </c>
       <c r="E6" s="1">
-        <v>117180</v>
+        <v>144100</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -3375,10 +3377,10 @@
         <v>195</v>
       </c>
       <c r="D7" s="1">
-        <v>116550</v>
+        <v>143200</v>
       </c>
       <c r="E7" s="1">
-        <v>122300</v>
+        <v>150350</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -3392,10 +3394,10 @@
         <v>193</v>
       </c>
       <c r="D8" s="1">
-        <v>184297</v>
+        <v>193500</v>
       </c>
       <c r="E8" s="1">
-        <v>204498</v>
+        <v>251300</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -3409,10 +3411,10 @@
         <v>194</v>
       </c>
       <c r="D9" s="1">
-        <v>184297</v>
+        <v>193500</v>
       </c>
       <c r="E9" s="1">
-        <v>204498</v>
+        <v>251300</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -3426,10 +3428,10 @@
         <v>195</v>
       </c>
       <c r="D10" s="1">
-        <v>194121</v>
+        <v>203850</v>
       </c>
       <c r="E10" s="1">
-        <v>208575</v>
+        <v>256250</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -3443,7 +3445,7 @@
         <v>193</v>
       </c>
       <c r="F11" s="1">
-        <v>64350</v>
+        <v>79500</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -3457,7 +3459,7 @@
         <v>194</v>
       </c>
       <c r="F12" s="1">
-        <v>64350</v>
+        <v>79500</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -3471,7 +3473,7 @@
         <v>195</v>
       </c>
       <c r="F13" s="1">
-        <v>67260</v>
+        <v>82600</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -3485,7 +3487,7 @@
         <v>193</v>
       </c>
       <c r="F14" s="1">
-        <v>133075</v>
+        <v>163500</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -3499,7 +3501,7 @@
         <v>194</v>
       </c>
       <c r="F15" s="1">
-        <v>133875</v>
+        <v>163500</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -3513,7 +3515,7 @@
         <v>195</v>
       </c>
       <c r="F16" s="1">
-        <v>145763</v>
+        <v>176500</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -3527,10 +3529,10 @@
         <v>193</v>
       </c>
       <c r="D17" s="1">
-        <v>174350</v>
+        <v>228900</v>
       </c>
       <c r="E17" s="1">
-        <v>174350</v>
+        <v>228900</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -3544,10 +3546,10 @@
         <v>194</v>
       </c>
       <c r="D18" s="1">
-        <v>174350</v>
+        <v>228900</v>
       </c>
       <c r="E18" s="1">
-        <v>174350</v>
+        <v>228900</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -3561,10 +3563,10 @@
         <v>195</v>
       </c>
       <c r="D19" s="1">
-        <v>186300</v>
+        <v>244500</v>
       </c>
       <c r="E19" s="1">
-        <v>186300</v>
+        <v>244500</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -3578,10 +3580,10 @@
         <v>193</v>
       </c>
       <c r="D20" s="1">
-        <v>206731</v>
+        <v>271400</v>
       </c>
       <c r="E20" s="1">
-        <v>206731</v>
+        <v>271400</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -3595,10 +3597,10 @@
         <v>194</v>
       </c>
       <c r="D21" s="1">
-        <v>206731</v>
+        <v>271400</v>
       </c>
       <c r="E21" s="1">
-        <v>206731</v>
+        <v>271400</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -3612,10 +3614,10 @@
         <v>195</v>
       </c>
       <c r="D22" s="1">
-        <v>208285</v>
+        <v>273400</v>
       </c>
       <c r="E22" s="1">
-        <v>208285</v>
+        <v>273400</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -3629,10 +3631,10 @@
         <v>193</v>
       </c>
       <c r="D23" s="1">
-        <v>271005</v>
+        <v>355700</v>
       </c>
       <c r="E23" s="1">
-        <v>271005</v>
+        <v>355700</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -3646,10 +3648,10 @@
         <v>194</v>
       </c>
       <c r="D24" s="1">
-        <v>271005</v>
+        <v>355700</v>
       </c>
       <c r="E24" s="1">
-        <v>271005</v>
+        <v>355700</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -3663,10 +3665,10 @@
         <v>195</v>
       </c>
       <c r="D25" s="1">
-        <v>286182</v>
+        <v>375600</v>
       </c>
       <c r="E25" s="1">
-        <v>286182</v>
+        <v>375600</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -6053,35 +6055,35 @@
         <v>56</v>
       </c>
       <c r="B55" s="2">
-        <f>B54*(1.05)</f>
+        <f t="shared" ref="B55:I55" si="0">B54*(1.05)</f>
         <v>306836.25</v>
       </c>
       <c r="C55" s="2">
-        <f>C54*(1.05)</f>
+        <f t="shared" si="0"/>
         <v>37687.65</v>
       </c>
       <c r="D55" s="2">
-        <f>D54*(1.05)</f>
+        <f t="shared" si="0"/>
         <v>71820</v>
       </c>
       <c r="E55" s="2">
-        <f>E54*(1.05)</f>
+        <f t="shared" si="0"/>
         <v>87088.05</v>
       </c>
       <c r="F55" s="2">
-        <f>F54*(1.05)</f>
+        <f t="shared" si="0"/>
         <v>100217.25</v>
       </c>
       <c r="G55" s="2">
-        <f>G54*(1.05)</f>
+        <f t="shared" si="0"/>
         <v>131964</v>
       </c>
       <c r="H55" s="2">
-        <f>H54*(1.05)</f>
+        <f t="shared" si="0"/>
         <v>413127.75</v>
       </c>
       <c r="I55" s="2">
-        <f>I54*(1.05)</f>
+        <f t="shared" si="0"/>
         <v>173365.5</v>
       </c>
     </row>
@@ -11220,10 +11222,10 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>25839</v>
+        <v>26974</v>
       </c>
       <c r="E2">
-        <v>28439</v>
+        <v>29689</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -11234,13 +11236,13 @@
         <v>105289</v>
       </c>
       <c r="C3">
-        <v>20196</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>24486</v>
+        <v>26974</v>
       </c>
       <c r="E3">
-        <v>26941</v>
+        <v>29689</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -11251,13 +11253,13 @@
         <v>140475</v>
       </c>
       <c r="C4">
-        <v>10098</v>
+        <v>10542</v>
       </c>
       <c r="D4">
-        <v>12243</v>
+        <v>12781</v>
       </c>
       <c r="E4">
-        <v>13471</v>
+        <v>14062</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -11268,13 +11270,13 @@
         <v>168040</v>
       </c>
       <c r="C5">
-        <v>10098</v>
+        <v>10542</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>13471</v>
+        <v>14062</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -11285,13 +11287,13 @@
         <v>157887</v>
       </c>
       <c r="C6">
-        <v>5643</v>
+        <v>5891</v>
       </c>
       <c r="D6">
-        <v>6798</v>
+        <v>7097</v>
       </c>
       <c r="E6">
-        <v>7484</v>
+        <v>7813</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -11302,13 +11304,13 @@
         <v>171861</v>
       </c>
       <c r="C7">
-        <v>5643</v>
+        <v>5891</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>7097</v>
       </c>
       <c r="E7">
-        <v>7484</v>
+        <v>7813</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
terminado, lo entrego hoy!
</commit_message>
<xml_diff>
--- a/backend/excel/catalogo.xlsx
+++ b/backend/excel/catalogo.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="10275" tabRatio="939" firstSheet="8" activeTab="13"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19395" windowHeight="10275" tabRatio="939" firstSheet="8" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="VENTANAS_HERRERO" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="281">
   <si>
     <t>MEDIDA</t>
   </si>
@@ -723,12 +723,6 @@
     <t>MOSQUITERO_FIJO</t>
   </si>
   <si>
-    <t>CAJON_BLOCK</t>
-  </si>
-  <si>
-    <t>CORTINAS</t>
-  </si>
-  <si>
     <t>PVC</t>
   </si>
   <si>
@@ -792,9 +786,6 @@
     <t>PUERTA_MOSQUITERO</t>
   </si>
   <si>
-    <t>6MM</t>
-  </si>
-  <si>
     <t>4+4</t>
   </si>
   <si>
@@ -835,14 +826,79 @@
   </si>
   <si>
     <t>GRANERO_ALUMINIO_SIN_HERRAJES</t>
+  </si>
+  <si>
+    <t>SUBITEM2</t>
+  </si>
+  <si>
+    <t>VARILLAS</t>
+  </si>
+  <si>
+    <t>CAJON_BLOCK_PRECIOS</t>
+  </si>
+  <si>
+    <t>CORTINAS_MODULO</t>
+  </si>
+  <si>
+    <t>LIVIANA_COMPLETA</t>
+  </si>
+  <si>
+    <t>LIVIANA_PANO_SOLO</t>
+  </si>
+  <si>
+    <t>REFORZADA_COMPLETA</t>
+  </si>
+  <si>
+    <t>REFORZADA_PANO_SOLO</t>
+  </si>
+  <si>
+    <t>SUPER_REFORZADA_COMPLETA</t>
+  </si>
+  <si>
+    <t>SUPER_REFORZADA_PANO_SOLO</t>
+  </si>
+  <si>
+    <t>BLANCO_COMPLETA</t>
+  </si>
+  <si>
+    <t>BLANCO_PANO_SOLO</t>
+  </si>
+  <si>
+    <t>SIMIL_MADERA_COMPLETA</t>
+  </si>
+  <si>
+    <t>SIMIL_MADERA_PANO_SOLO</t>
+  </si>
+  <si>
+    <t>BARRA_ANTIPANICO</t>
+  </si>
+  <si>
+    <t>LAMINADO</t>
+  </si>
+  <si>
+    <t>TEMPLADO</t>
+  </si>
+  <si>
+    <t>REFLECTIVO</t>
+  </si>
+  <si>
+    <t>LOW_E</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -870,13 +926,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3278,7 +3340,7 @@
         <v>190</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -3673,10 +3735,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>193</v>
@@ -3687,10 +3749,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>194</v>
@@ -3701,10 +3763,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>195</v>
@@ -3715,10 +3777,10 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>193</v>
@@ -3729,10 +3791,10 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>194</v>
@@ -3743,10 +3805,10 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>195</v>
@@ -3757,10 +3819,10 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>263</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>193</v>
@@ -3771,10 +3833,10 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>263</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>194</v>
@@ -3785,10 +3847,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>263</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>195</v>
@@ -3799,10 +3861,10 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>193</v>
@@ -3813,10 +3875,10 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>194</v>
@@ -3827,10 +3889,10 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>195</v>
@@ -3846,90 +3908,109 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="D4" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="D5" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="D6" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="D7" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>218</v>
       </c>
@@ -3939,11 +4020,11 @@
       <c r="C8" t="s">
         <v>220</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>10685</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>218</v>
       </c>
@@ -3953,33 +4034,33 @@
       <c r="C9" t="s">
         <v>221</v>
       </c>
-      <c r="D9">
-        <v>20505</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9">
+        <v>18080</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>218</v>
       </c>
       <c r="B10" t="s">
         <v>222</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>7400</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>218</v>
       </c>
       <c r="B11" t="s">
         <v>223</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>4200</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>218</v>
       </c>
@@ -3989,11 +4070,11 @@
       <c r="C12" t="s">
         <v>220</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>13517</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>218</v>
       </c>
@@ -4003,422 +4084,647 @@
       <c r="C13" t="s">
         <v>221</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>20505</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>218</v>
       </c>
       <c r="B14" t="s">
         <v>225</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>5905</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>218</v>
       </c>
       <c r="B15" t="s">
-        <v>226</v>
-      </c>
-      <c r="D15">
-        <v>48364</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>263</v>
+      </c>
+      <c r="E15">
+        <v>18500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>218</v>
       </c>
       <c r="B16" t="s">
-        <v>227</v>
-      </c>
-      <c r="D16">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+      <c r="E16">
+        <v>48364</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>218</v>
       </c>
       <c r="B17" t="s">
-        <v>228</v>
+        <v>264</v>
       </c>
       <c r="C17" t="s">
-        <v>229</v>
-      </c>
-      <c r="D17">
-        <v>18500</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>227</v>
+      </c>
+      <c r="E17">
+        <v>280585</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>218</v>
       </c>
       <c r="B18" t="s">
-        <v>228</v>
+        <v>264</v>
       </c>
       <c r="C18" t="s">
         <v>190</v>
       </c>
-      <c r="D18">
-        <v>42000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="E18">
+        <v>346865</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>218</v>
+      </c>
+      <c r="B20" t="s">
+        <v>265</v>
+      </c>
+      <c r="C20" t="s">
+        <v>227</v>
+      </c>
+      <c r="D20" t="s">
+        <v>266</v>
+      </c>
+      <c r="E20">
+        <v>30208</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>218</v>
+      </c>
+      <c r="B21" t="s">
+        <v>265</v>
+      </c>
+      <c r="C21" t="s">
+        <v>227</v>
+      </c>
+      <c r="D21" t="s">
+        <v>267</v>
+      </c>
+      <c r="E21">
+        <v>23180</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>218</v>
+      </c>
+      <c r="B22" t="s">
+        <v>265</v>
+      </c>
+      <c r="C22" t="s">
+        <v>227</v>
+      </c>
+      <c r="D22" t="s">
+        <v>268</v>
+      </c>
+      <c r="E22">
+        <v>37410</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>218</v>
+      </c>
+      <c r="B23" t="s">
+        <v>265</v>
+      </c>
+      <c r="C23" t="s">
+        <v>227</v>
+      </c>
+      <c r="D23" t="s">
+        <v>269</v>
+      </c>
+      <c r="E23">
+        <v>28263</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>218</v>
+      </c>
+      <c r="B24" t="s">
+        <v>265</v>
+      </c>
+      <c r="C24" t="s">
+        <v>227</v>
+      </c>
+      <c r="D24" t="s">
+        <v>270</v>
+      </c>
+      <c r="E24">
+        <v>52671</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>218</v>
+      </c>
+      <c r="B25" t="s">
+        <v>265</v>
+      </c>
+      <c r="C25" t="s">
+        <v>227</v>
+      </c>
+      <c r="D25" t="s">
+        <v>271</v>
+      </c>
+      <c r="E25">
+        <v>39099</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>218</v>
+      </c>
+      <c r="B27" t="s">
+        <v>265</v>
+      </c>
+      <c r="C27" t="s">
+        <v>190</v>
+      </c>
+      <c r="D27" t="s">
+        <v>272</v>
+      </c>
+      <c r="E27">
+        <v>188750</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>218</v>
+      </c>
+      <c r="B28" t="s">
+        <v>265</v>
+      </c>
+      <c r="C28" t="s">
+        <v>190</v>
+      </c>
+      <c r="D28" t="s">
+        <v>273</v>
+      </c>
+      <c r="E28">
+        <v>139851</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>218</v>
+      </c>
+      <c r="B29" t="s">
+        <v>265</v>
+      </c>
+      <c r="C29" t="s">
+        <v>190</v>
+      </c>
+      <c r="D29" t="s">
+        <v>274</v>
+      </c>
+      <c r="E29">
+        <v>204007</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>218</v>
+      </c>
+      <c r="B30" t="s">
+        <v>265</v>
+      </c>
+      <c r="C30" t="s">
+        <v>190</v>
+      </c>
+      <c r="D30" t="s">
+        <v>275</v>
+      </c>
+      <c r="E30">
+        <v>155108</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>228</v>
+      </c>
+      <c r="B31" t="s">
+        <v>229</v>
+      </c>
+      <c r="E31">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>228</v>
+      </c>
+      <c r="B32" t="s">
         <v>230</v>
       </c>
-      <c r="B19" t="s">
+      <c r="E32">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>228</v>
+      </c>
+      <c r="B33" t="s">
         <v>231</v>
       </c>
-      <c r="D19">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>230</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="E33">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>228</v>
+      </c>
+      <c r="B34" t="s">
         <v>232</v>
       </c>
-      <c r="D20">
+      <c r="E34">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>228</v>
+      </c>
+      <c r="B35" t="s">
+        <v>233</v>
+      </c>
+      <c r="E35">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>228</v>
+      </c>
+      <c r="B36" t="s">
+        <v>234</v>
+      </c>
+      <c r="E36">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>228</v>
+      </c>
+      <c r="B37" t="s">
+        <v>235</v>
+      </c>
+      <c r="E37">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>236</v>
+      </c>
+      <c r="B38" t="s">
+        <v>237</v>
+      </c>
+      <c r="E38">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>236</v>
+      </c>
+      <c r="B39" t="s">
+        <v>238</v>
+      </c>
+      <c r="E39">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>239</v>
+      </c>
+      <c r="B40" t="s">
+        <v>153</v>
+      </c>
+      <c r="E40">
+        <v>550000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>239</v>
+      </c>
+      <c r="B41" t="s">
+        <v>240</v>
+      </c>
+      <c r="E41">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>239</v>
+      </c>
+      <c r="B42" t="s">
+        <v>241</v>
+      </c>
+      <c r="E42">
+        <v>850000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>239</v>
+      </c>
+      <c r="B43" t="s">
+        <v>242</v>
+      </c>
+      <c r="E43">
+        <v>600000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>239</v>
+      </c>
+      <c r="B44" t="s">
+        <v>243</v>
+      </c>
+      <c r="E44">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>239</v>
+      </c>
+      <c r="B45" t="s">
+        <v>276</v>
+      </c>
+      <c r="E45">
+        <v>225000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>239</v>
+      </c>
+      <c r="B46" t="s">
+        <v>244</v>
+      </c>
+      <c r="C46" t="s">
+        <v>220</v>
+      </c>
+      <c r="E46">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>239</v>
+      </c>
+      <c r="B47" t="s">
+        <v>244</v>
+      </c>
+      <c r="C47" t="s">
+        <v>221</v>
+      </c>
+      <c r="E47">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>239</v>
+      </c>
+      <c r="B48" t="s">
+        <v>245</v>
+      </c>
+      <c r="E48">
+        <v>11500</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>239</v>
+      </c>
+      <c r="B49" t="s">
+        <v>246</v>
+      </c>
+      <c r="C49" t="s">
+        <v>220</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>239</v>
+      </c>
+      <c r="B50" t="s">
+        <v>246</v>
+      </c>
+      <c r="C50" t="s">
+        <v>221</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>247</v>
+      </c>
+      <c r="B51">
+        <v>80</v>
+      </c>
+      <c r="E51">
+        <v>101970</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>247</v>
+      </c>
+      <c r="B52">
+        <v>90</v>
+      </c>
+      <c r="E52">
+        <v>112167</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>4</v>
+      </c>
+      <c r="B53" t="s">
+        <v>60</v>
+      </c>
+      <c r="E53">
+        <v>29500</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>4</v>
+      </c>
+      <c r="B54">
+        <v>4</v>
+      </c>
+      <c r="E54">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>4</v>
+      </c>
+      <c r="B55">
+        <v>5</v>
+      </c>
+      <c r="E55">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>4</v>
+      </c>
+      <c r="B56">
+        <v>6</v>
+      </c>
+      <c r="E56">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>4</v>
+      </c>
+      <c r="B57">
+        <v>8</v>
+      </c>
+      <c r="E57">
         <v>45000</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>230</v>
-      </c>
-      <c r="B21" t="s">
-        <v>233</v>
-      </c>
-      <c r="D21">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>230</v>
-      </c>
-      <c r="B22" t="s">
-        <v>234</v>
-      </c>
-      <c r="D22">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B23" t="s">
-        <v>235</v>
-      </c>
-      <c r="D23">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>230</v>
-      </c>
-      <c r="B24" t="s">
-        <v>236</v>
-      </c>
-      <c r="D24">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>230</v>
-      </c>
-      <c r="B25" t="s">
-        <v>237</v>
-      </c>
-      <c r="D25">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>238</v>
-      </c>
-      <c r="B26" t="s">
-        <v>239</v>
-      </c>
-      <c r="D26">
-        <v>16500</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>238</v>
-      </c>
-      <c r="B27" t="s">
-        <v>240</v>
-      </c>
-      <c r="D27">
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>241</v>
-      </c>
-      <c r="B28" t="s">
-        <v>153</v>
-      </c>
-      <c r="D28">
-        <v>550000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>241</v>
-      </c>
-      <c r="B29" t="s">
-        <v>242</v>
-      </c>
-      <c r="D29">
-        <v>400000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>241</v>
-      </c>
-      <c r="B30" t="s">
-        <v>243</v>
-      </c>
-      <c r="D30">
-        <v>850000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>241</v>
-      </c>
-      <c r="B31" t="s">
-        <v>244</v>
-      </c>
-      <c r="D31">
-        <v>800000</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>241</v>
-      </c>
-      <c r="B32" t="s">
-        <v>245</v>
-      </c>
-      <c r="D32">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>241</v>
-      </c>
-      <c r="B33" t="s">
-        <v>246</v>
-      </c>
-      <c r="C33" t="s">
-        <v>220</v>
-      </c>
-      <c r="D33">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>241</v>
-      </c>
-      <c r="B34" t="s">
-        <v>246</v>
-      </c>
-      <c r="C34" t="s">
-        <v>221</v>
-      </c>
-      <c r="D34">
-        <v>12000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>241</v>
-      </c>
-      <c r="B35" t="s">
-        <v>247</v>
-      </c>
-      <c r="D35">
-        <v>11500</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>241</v>
-      </c>
-      <c r="B36" t="s">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>4</v>
+      </c>
+      <c r="B58">
+        <v>10</v>
+      </c>
+      <c r="E58">
+        <v>67000</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>4</v>
+      </c>
+      <c r="B59" t="s">
         <v>248</v>
       </c>
-      <c r="C36" t="s">
-        <v>220</v>
-      </c>
-      <c r="D36">
+      <c r="E59">
+        <v>59000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>4</v>
+      </c>
+      <c r="B60" t="s">
+        <v>249</v>
+      </c>
+      <c r="E60">
+        <v>79000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>4</v>
+      </c>
+      <c r="B61" t="s">
+        <v>61</v>
+      </c>
+      <c r="E61">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>241</v>
-      </c>
-      <c r="B37" t="s">
-        <v>248</v>
-      </c>
-      <c r="C37" t="s">
-        <v>221</v>
-      </c>
-      <c r="D37">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>4</v>
+      </c>
+      <c r="B62" t="s">
+        <v>277</v>
+      </c>
+      <c r="E62">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>249</v>
-      </c>
-      <c r="B38">
-        <v>80</v>
-      </c>
-      <c r="D38">
-        <v>101970</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>249</v>
-      </c>
-      <c r="B39">
-        <v>90</v>
-      </c>
-      <c r="D39">
-        <v>112167</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>4</v>
       </c>
-      <c r="B40" t="s">
-        <v>57</v>
-      </c>
-      <c r="D40">
-        <v>16459</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="B63" t="s">
+        <v>278</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>4</v>
       </c>
-      <c r="B41" t="s">
-        <v>58</v>
-      </c>
-      <c r="D41">
-        <v>21250</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="B64" t="s">
+        <v>62</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>4</v>
       </c>
-      <c r="B42" t="s">
-        <v>59</v>
-      </c>
-      <c r="D42">
-        <v>27169</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="B65" t="s">
+        <v>279</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>4</v>
       </c>
-      <c r="B43" t="s">
-        <v>250</v>
-      </c>
-      <c r="D43">
-        <v>33410</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>4</v>
-      </c>
-      <c r="B44" t="s">
-        <v>63</v>
-      </c>
-      <c r="D44">
-        <v>27012</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>4</v>
-      </c>
-      <c r="B45" t="s">
-        <v>62</v>
-      </c>
-      <c r="D45">
-        <v>60797</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>4</v>
-      </c>
-      <c r="B46" t="s">
-        <v>60</v>
-      </c>
-      <c r="D46">
-        <v>65546</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>4</v>
-      </c>
-      <c r="B47" t="s">
-        <v>251</v>
-      </c>
-      <c r="D47">
-        <v>73221</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>4</v>
-      </c>
-      <c r="B48" t="s">
-        <v>252</v>
-      </c>
-      <c r="D48">
-        <v>88575</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>4</v>
-      </c>
-      <c r="B49" t="s">
-        <v>61</v>
-      </c>
-      <c r="D49">
-        <v>12600</v>
+      <c r="B66" t="s">
+        <v>280</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4433,7 +4739,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B1" t="s">
         <v>205</v>
@@ -4444,12 +4750,12 @@
         <v>215</v>
       </c>
       <c r="B2" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -4457,18 +4763,18 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B4" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B5" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
genera listas y un millon de bugs...
</commit_message>
<xml_diff>
--- a/backend/excel/catalogo.xlsx
+++ b/backend/excel/catalogo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\German\Documents\sebamarapp\backend\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57120DDC-16E1-4A38-B169-680F689B46F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C974BA-FD53-48C5-8805-2FD080D941A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" tabRatio="939" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1258,7 +1258,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="1">
-        <v>26000</v>
+        <v>26195</v>
       </c>
       <c r="C2" s="1">
         <v>7179</v>
@@ -2177,6 +2177,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
3h 3g, v/r, y un par de cosas mas
</commit_message>
<xml_diff>
--- a/backend/excel/catalogo.xlsx
+++ b/backend/excel/catalogo.xlsx
@@ -3364,10 +3364,10 @@
         <v>193</v>
       </c>
       <c r="D2" s="1">
-        <v>76300</v>
+        <v>80200</v>
       </c>
       <c r="E2" s="1">
-        <v>81100</v>
+        <v>85200</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3381,10 +3381,10 @@
         <v>194</v>
       </c>
       <c r="D3" s="1">
-        <v>76300</v>
+        <v>80200</v>
       </c>
       <c r="E3" s="1">
-        <v>81100</v>
+        <v>85200</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -3398,10 +3398,10 @@
         <v>195</v>
       </c>
       <c r="D4" s="1">
-        <v>81100</v>
+        <v>85200</v>
       </c>
       <c r="E4" s="1">
-        <v>86112</v>
+        <v>90420</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3517,7 +3517,7 @@
         <v>193</v>
       </c>
       <c r="F11" s="1">
-        <v>79500</v>
+        <v>83500</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -3531,7 +3531,7 @@
         <v>194</v>
       </c>
       <c r="F12" s="1">
-        <v>79500</v>
+        <v>83500</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -3545,7 +3545,7 @@
         <v>195</v>
       </c>
       <c r="F13" s="1">
-        <v>82600</v>
+        <v>86730</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -3601,10 +3601,10 @@
         <v>193</v>
       </c>
       <c r="D17" s="1">
-        <v>228900</v>
+        <v>240345</v>
       </c>
       <c r="E17" s="1">
-        <v>228900</v>
+        <v>240345</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -3618,10 +3618,10 @@
         <v>194</v>
       </c>
       <c r="D18" s="1">
-        <v>228900</v>
+        <v>240345</v>
       </c>
       <c r="E18" s="1">
-        <v>228900</v>
+        <v>240345</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -3635,10 +3635,10 @@
         <v>195</v>
       </c>
       <c r="D19" s="1">
-        <v>244500</v>
+        <v>256725</v>
       </c>
       <c r="E19" s="1">
-        <v>244500</v>
+        <v>256725</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>